<commit_message>
LOGLAMA İŞLEMİN KALDIRILMASI. MÜFREDATLARIN 4DERLİ OLARAK DEĞİŞTİRİLMESİ.
</commit_message>
<xml_diff>
--- a/data/2022_Mufredat.xlsx
+++ b/data/2022_Mufredat.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dadil\Documents\Yazilimsal_Projeler\BitirmeProje\Adil_Secmeli_Python\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E52FCBAE-1584-4445-A616-D774981C2A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD89A990-1287-4E98-AA52-3002029AF24D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="60">
   <si>
     <t>ID</t>
   </si>
@@ -49,9 +49,6 @@
     <t>Seçmeli Ders 4</t>
   </si>
   <si>
-    <t>Seçmeli Ders 5</t>
-  </si>
-  <si>
     <t>Tıp Fakültesi</t>
   </si>
   <si>
@@ -73,9 +70,6 @@
     <t>Toplum ve Kültürü Anlamak</t>
   </si>
   <si>
-    <t>Kariyer Planlama</t>
-  </si>
-  <si>
     <t>Bulut Bilişim Uygulamaları</t>
   </si>
   <si>
@@ -88,9 +82,6 @@
     <t>Mobil Programlama</t>
   </si>
   <si>
-    <t>Siber Güvenlik ve Kriptoloji</t>
-  </si>
-  <si>
     <t>Gömülü Sistemler - I</t>
   </si>
   <si>
@@ -103,9 +94,6 @@
     <t>FPGA İle Gömülü Sistem Tasarımı</t>
   </si>
   <si>
-    <t>Haberleşme Elektroniği</t>
-  </si>
-  <si>
     <t>Endüstri 4.0 ve Dijital Dönüşüm</t>
   </si>
   <si>
@@ -118,9 +106,6 @@
     <t>Karar Destek Sistemleri</t>
   </si>
   <si>
-    <t>İnsan Kaynakları Yönetimi</t>
-  </si>
-  <si>
     <t>Hemşirelik</t>
   </si>
   <si>
@@ -136,9 +121,6 @@
     <t>Diyaliz Hemşireliği</t>
   </si>
   <si>
-    <t>İlk Yardım</t>
-  </si>
-  <si>
     <t>Ebelik</t>
   </si>
   <si>
@@ -154,9 +136,6 @@
     <t>Perinatal Ruh Sağlığı</t>
   </si>
   <si>
-    <t>Adli Ebelik</t>
-  </si>
-  <si>
     <t>Sporcu Sağlığı ve Rehabilitasyonu</t>
   </si>
   <si>
@@ -169,9 +148,6 @@
     <t>Tele-Rehabilitasyon</t>
   </si>
   <si>
-    <t>Yoga ve Pilates</t>
-  </si>
-  <si>
     <t>Gastronomi</t>
   </si>
   <si>
@@ -187,9 +163,6 @@
     <t>Antik Mutfaklar</t>
   </si>
   <si>
-    <t>Gastronomi ve Sanat</t>
-  </si>
-  <si>
     <t>İlahiyat Fakültesi</t>
   </si>
   <si>
@@ -206,9 +179,6 @@
   </si>
   <si>
     <t>Kur'an-ı Kerim Talimi</t>
-  </si>
-  <si>
-    <t>Medeniyetler ve Küresel Karşılaşmalar</t>
   </si>
   <si>
     <t>Mühendislik ve Doğa Bilimleri Fakültesi</t>
@@ -548,297 +518,277 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
+      <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>11</v>
-      </c>
       <c r="D2" s="3">
         <v>2022</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="D3" s="3">
         <v>2022</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>22</v>
-      </c>
+      <c r="J3" s="1"/>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="D4" s="3">
         <v>2022</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="D5" s="3">
         <v>2022</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>32</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="J5" s="1"/>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D6" s="3">
         <v>2022</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>38</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="J6" s="1"/>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D7" s="3">
         <v>2022</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>44</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="J7" s="1"/>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="D8" s="3">
         <v>2022</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>49</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="J8" s="1"/>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="2">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="D9" s="3">
         <v>2022</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>55</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="J9" s="1"/>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D10" s="3">
         <v>2022</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>62</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="J10" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>